<commit_message>
Auto update (2026-05-08 17:51:41) | Files: node/suivi_site_20260508.xlsx suivi_site.xlsx
</commit_message>
<xml_diff>
--- a/node/suivi_site_20260508.xlsx
+++ b/node/suivi_site_20260508.xlsx
@@ -442,7 +442,7 @@
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,7 +563,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1 days 01:13:37</t>
+          <t>25:30:23</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0 days 08:31:50</t>
+          <t>08:48:36</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0 days 08:31:50</t>
+          <t>08:48:36</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0 days 08:31:50</t>
+          <t>08:48:36</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0 days 08:31:07</t>
+          <t>08:47:53</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0 days 07:29:16</t>
+          <t>07:46:02</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0 days 02:56:21</t>
+          <t>03:13:07</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0 days 02:55:21</t>
+          <t>03:12:07</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0 days 02:55:03</t>
+          <t>03:11:49</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0 days 02:04:21</t>
+          <t>02:21:07</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0 days 02:04:21</t>
+          <t>02:21:07</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0 days 01:35:03</t>
+          <t>01:51:49</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0 days 01:30:41</t>
+          <t>01:47:27</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0 days 01:30:41</t>
+          <t>01:47:27</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0 days 01:30:41</t>
+          <t>01:47:27</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0 days 01:30:41</t>
+          <t>01:47:27</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0 days 01:30:41</t>
+          <t>01:47:27</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0 days 01:23:20</t>
+          <t>01:40:06</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0 days 00:40:11</t>
+          <t>00:56:57</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0 days 00:38:41</t>
+          <t>00:55:27</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0 days 00:34:41</t>
+          <t>00:51:27</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1 days 01:56:50</t>
+          <t>26:13:36</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1 days 01:56:48</t>
+          <t>26:13:34</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0 days 05:56:55</t>
+          <t>06:13:41</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0 days 02:21:36</t>
+          <t>02:38:22</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0 days 02:12:49</t>
+          <t>02:29:35</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0 days 02:06:47</t>
+          <t>02:23:33</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0 days 01:49:02</t>
+          <t>02:05:48</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0 days 00:57:12</t>
+          <t>01:13:58</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0 days 00:50:10</t>
+          <t>01:06:56</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0 days 00:39:43</t>
+          <t>00:56:29</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0 days 00:39:37</t>
+          <t>00:56:23</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0 days 00:36:27</t>
+          <t>00:53:13</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0 days 00:57:16</t>
+          <t>01:14:02</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0 days 00:33:41</t>
+          <t>00:50:27</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0 days 08:29:34</t>
+          <t>08:46:20</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0 days 08:34:22</t>
+          <t>08:51:08</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0 days 01:07:04</t>
+          <t>01:23:50</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0 days 13:50:23</t>
+          <t>14:07:09</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0 days 13:49:57</t>
+          <t>14:06:43</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0 days 09:15:25</t>
+          <t>09:32:11</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0 days 09:14:58</t>
+          <t>09:31:44</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0 days 08:28:47</t>
+          <t>08:45:33</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0 days 08:27:26</t>
+          <t>08:44:12</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3178,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0 days 08:26:52</t>
+          <t>08:43:38</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0 days 08:24:57</t>
+          <t>08:41:43</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0 days 06:10:44</t>
+          <t>06:27:30</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0 days 06:10:29</t>
+          <t>06:27:15</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>0 days 06:10:24</t>
+          <t>06:27:10</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>0 days 06:10:12</t>
+          <t>06:26:58</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>0 days 04:56:58</t>
+          <t>05:13:44</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0 days 04:55:48</t>
+          <t>05:12:34</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>0 days 02:50:43</t>
+          <t>03:07:29</t>
         </is>
       </c>
     </row>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>0 days 02:50:36</t>
+          <t>03:07:22</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>0 days 02:00:21</t>
+          <t>02:17:07</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>0 days 01:59:38</t>
+          <t>02:16:24</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>0 days 01:31:42</t>
+          <t>01:48:28</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>0 days 01:30:53</t>
+          <t>01:47:39</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>0 days 01:30:52</t>
+          <t>01:47:38</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>0 days 01:28:23</t>
+          <t>01:45:09</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>0 days 01:27:57</t>
+          <t>01:44:43</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>0 days 01:27:48</t>
+          <t>01:44:34</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0 days 01:27:33</t>
+          <t>01:44:19</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>0 days 01:27:22</t>
+          <t>01:44:08</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>0 days 01:27:20</t>
+          <t>01:44:06</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>0 days 01:27:18</t>
+          <t>01:44:04</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>0 days 01:26:53</t>
+          <t>01:43:39</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>0 days 01:26:36</t>
+          <t>01:43:22</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4563,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>0 days 01:26:33</t>
+          <t>01:43:19</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>0 days 01:26:19</t>
+          <t>01:43:05</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>0 days 01:26:08</t>
+          <t>01:42:54</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>0 days 01:20:30</t>
+          <t>01:37:16</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>0 days 01:19:54</t>
+          <t>01:36:40</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>0 days 01:18:20</t>
+          <t>01:35:06</t>
         </is>
       </c>
     </row>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>0 days 01:18:00</t>
+          <t>01:34:46</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>0 days 00:56:17</t>
+          <t>01:13:03</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>0 days 00:56:17</t>
+          <t>01:13:03</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>1 days 01:53:21</t>
+          <t>26:10:07</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>1 days 01:53:21</t>
+          <t>26:10:07</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>0 days 05:53:56</t>
+          <t>06:10:42</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>0 days 02:18:20</t>
+          <t>02:35:06</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5318,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>0 days 02:09:37</t>
+          <t>02:26:23</t>
         </is>
       </c>
     </row>
@@ -5378,7 +5378,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>0 days 01:45:31</t>
+          <t>02:02:17</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>0 days 00:53:52</t>
+          <t>01:10:38</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>0 days 00:53:44</t>
+          <t>01:10:30</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>0 days 00:46:52</t>
+          <t>01:03:38</t>
         </is>
       </c>
     </row>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>0 days 00:36:33</t>
+          <t>00:53:19</t>
         </is>
       </c>
     </row>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>0 days 00:36:33</t>
+          <t>00:53:19</t>
         </is>
       </c>
     </row>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>0 days 00:33:31</t>
+          <t>00:50:17</t>
         </is>
       </c>
     </row>
@@ -5798,7 +5798,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>1 days 00:14:04</t>
+          <t>24:30:50</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>0 days 13:49:18</t>
+          <t>14:06:04</t>
         </is>
       </c>
     </row>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>0 days 08:27:57</t>
+          <t>08:44:43</t>
         </is>
       </c>
     </row>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>0 days 08:32:55</t>
+          <t>08:49:41</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>0 days 08:27:57</t>
+          <t>08:44:43</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>0 days 08:26:30</t>
+          <t>08:43:16</t>
         </is>
       </c>
     </row>
@@ -6158,7 +6158,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>0 days 06:15:23</t>
+          <t>06:32:09</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>0 days 06:15:23</t>
+          <t>06:32:09</t>
         </is>
       </c>
     </row>
@@ -6278,7 +6278,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>0 days 05:01:38</t>
+          <t>05:18:24</t>
         </is>
       </c>
     </row>
@@ -6338,7 +6338,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>0 days 02:56:14</t>
+          <t>03:13:00</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6398,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>0 days 02:02:35</t>
+          <t>02:19:21</t>
         </is>
       </c>
     </row>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>0 days 01:21:02</t>
+          <t>01:37:48</t>
         </is>
       </c>
     </row>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>0 days 01:32:30</t>
+          <t>01:49:16</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>0 days 01:28:58</t>
+          <t>01:45:44</t>
         </is>
       </c>
     </row>
@@ -6638,7 +6638,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>0 days 01:25:48</t>
+          <t>01:42:34</t>
         </is>
       </c>
     </row>
@@ -6698,7 +6698,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>0 days 01:25:43</t>
+          <t>01:42:29</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>0 days 01:25:40</t>
+          <t>01:42:26</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>0 days 01:24:23</t>
+          <t>01:41:09</t>
         </is>
       </c>
     </row>
@@ -6878,7 +6878,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>0 days 01:24:21</t>
+          <t>01:41:07</t>
         </is>
       </c>
     </row>
@@ -6938,7 +6938,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>0 days 01:01:40</t>
+          <t>01:18:26</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>0 days 00:38:06</t>
+          <t>00:54:52</t>
         </is>
       </c>
     </row>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>1 days 01:58:11</t>
+          <t>26:14:57</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>1 days 01:58:11</t>
+          <t>26:14:57</t>
         </is>
       </c>
     </row>
@@ -7178,7 +7178,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>0 days 05:58:16</t>
+          <t>06:15:02</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7238,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>0 days 02:23:00</t>
+          <t>02:39:46</t>
         </is>
       </c>
     </row>
@@ -7298,7 +7298,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>0 days 02:14:09</t>
+          <t>02:30:55</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7358,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>0 days 01:50:19</t>
+          <t>02:07:05</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>0 days 00:58:37</t>
+          <t>01:15:23</t>
         </is>
       </c>
     </row>
@@ -7478,7 +7478,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>0 days 00:51:30</t>
+          <t>01:08:16</t>
         </is>
       </c>
     </row>
@@ -7538,7 +7538,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>0 days 00:41:04</t>
+          <t>00:57:50</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>0 days 00:40:59</t>
+          <t>00:57:45</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>0 days 00:37:53</t>
+          <t>00:54:39</t>
         </is>
       </c>
     </row>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>0 days 00:58:36</t>
+          <t>01:15:22</t>
         </is>
       </c>
     </row>
@@ -7778,7 +7778,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>0 days 00:35:07</t>
+          <t>00:51:53</t>
         </is>
       </c>
     </row>

</xml_diff>